<commit_message>
chore: replace Excel tracker with HTML tracker
</commit_message>
<xml_diff>
--- a/master-seo-map.xlsx
+++ b/master-seo-map.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master SEO Map" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cannibalization Resolution" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hub-Spoke Architecture" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unmapped Clusters" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Order" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERP Intelligence" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hub-Spoke Architecture" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unmapped Clusters" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Order" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master SEO Map'!$A$1:$Q$29</definedName>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +42,11 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +108,11 @@
         <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDDDDD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -131,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -182,6 +191,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -732,7 +745,7 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Write final conversion-focused content. This page OWNS "ai visibility audit" cluster. Blog tools-vs-audit must NOT target this keyword — it should link here instead.</t>
+          <t>Write final conversion-focused content. Per live SERP: direct competitors include LLMClicks.ai and AI Search Engineers (both sell same product). Differentiation: consultant-led (not agency), Canadian, with public case study (HomeCalc), transparent methodology. Consider future PR play: AI Search Engineers got Morningstar coverage by publishing 'findings from 50+ audits' style PR.</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
@@ -1396,7 +1409,7 @@
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>Wire internal links to ALL child service pages and blog spokes. This is the topical authority anchor.</t>
+          <t>Add case study proof links. Strengthen local-intent signals. Per live SERP: direct Canadian competitors are dNOVO Group (Toronto), Chief AI Advisors (Victoria BC), Pro Marketer. Wedge: personal brand (Hami the person, photo, bio) vs agency competitors. Toronto-specific case study (HomeCalc) is a strong signal. Add local schema (LocalBusiness or Person + areaServed=Canada/Toronto). Set up Google Business Profile if not done.</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
@@ -1645,7 +1658,7 @@
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Focus on "what is" definition angle. TL;DR box for AI extraction. Do NOT compete with hub on broad "ai visibility" — this is the explainer.</t>
+          <t>Comparison post. Per live SERP: authority sites dominate (Yext, Jasper, DMI). To win positions 4-8: 3-column comparison table, simple visual, FAQPage schema, named author. Each section links to the corresponding service page (AEO/GEO/SEO).</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
@@ -2050,7 +2063,7 @@
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>None (checker intent is distinct from tools-list intent)</t>
+          <t>Listicle format overlaps with /blog/best-ai-visibility-tools/ — but distinct: 'checkers' = free one-off tests (this page); 'tools/trackers' = paid ongoing software (best-tools page). Both pages must clearly state their angle in H1 + intro.</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
@@ -2060,7 +2073,7 @@
       </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
-          <t>Checker-intent post. Funnels to audit as the "done for you" option.</t>
+          <t>STRATEGIC PIVOT (per live SERP check): SERP for 'how to check ai visibility' is dominated by FREE CHECKER TOOLS, not how-to blog posts. Reframe this post as 'I Tested 10 Free AI Visibility Checkers — Here's What Each Actually Found' — a tested-tools listicle (not a pure instructional). Ends with 'or skip the tools, get a professional audit' CTA → audit page. Same URL, listicle angle.</t>
         </is>
       </c>
       <c r="Q18" s="8" t="inlineStr">
@@ -2226,7 +2239,7 @@
       </c>
       <c r="P20" s="10" t="inlineStr">
         <is>
-          <t>HIGHEST volume page (10,830). Tool listicle. CTA at bottom: "tools show you data, an audit tells you what to do." Links to audit.</t>
+          <t>HIGHEST volume page (10,830). Tool listicle. Per live SERP: Profound owns #1 with self-promotional listicle. Zapier (huge DR) ranks. EEAT is the wedge: named author bio at top, 'I'm an independent consultant, I don't sell these tools' methodology blurb, ratings table, transparent criteria. CTA at bottom: 'tools show you data, an audit tells you what to do.' Links to audit.</t>
         </is>
       </c>
       <c r="Q20" s="10" t="inlineStr">
@@ -3252,6 +3265,264 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>SERP Intent (Live)</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Top Competitors</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Risk / Opportunity</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Strategy Impact on Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>ai brand visibility tracking</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="n">
+        <v>5550</v>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>Tool/product pages dominate. Listicles in pos 5-9.</t>
+        </is>
+      </c>
+      <c r="E2" s="19" t="inlineStr">
+        <is>
+          <t>Ubersuggest, Peec AI, Otterly, Authoritas, SE Visible, Profound, Position.digital, WPEngine</t>
+        </is>
+      </c>
+      <c r="F2" s="19" t="inlineStr">
+        <is>
+          <t>Risk: SERP wants tools, not blogs. Opportunity: independent-consultant review angle is differentiator.</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>/blog/best-ai-visibility-tools/ MUST lean hard on EEAT: named author, transparent methodology, 'I tested these for clients' framing. Comparison table. NOT just an SEO listicle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>best ai visibility tools 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>Pure listicle SERP. Mix of tool vendors writing their own listicles + neutral roundups.</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>Profound (own blog ranks #1 — self-promotional listicle), Evertune, Rankability, Wellows, Nick Lafferty, Amplitude, Visiblie, SE Ranking, Zapier</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Risk: Profound owns #1 with self-promotional listicle (smart play). Zapier has massive DR. Opportunity: vendor-independent angle.</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>Same as #1 — EEAT critical. Consider: a methodology blurb at top ('I'm a consultant, I don't sell these tools, here's how I rated them').</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>ai visibility audit</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>70</v>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Mix of service pages + blog posts. Audit-as-a-service is a recognized product category.</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>Ahrefs (blog), AI Search Engineers (service + PR releases on Morningstar), LLMClicks (service page selling audits), SearchEngineJournal (questions list)</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Risk: LLMClicks.ai and AI Search Engineers are direct competitors selling the SAME product. Opportunity: AI Search Engineers got Morningstar PR — replicate.</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>/ai-visibility/ai-visibility-audit/ needs explicit differentiation: consultant-led (not agency), Canadian, with public case study (HomeCalc). Consider PR play: publish '50 audits done — findings' style report when have volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>aeo vs geo vs seo</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>310</v>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>100% explainer-blog SERP. Authority-site dominated.</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Digiday, Yext, Jasper, Hibu, DMI, LinkedIn, SearchEnginePeople</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Risk: authority sites (Yext, Jasper, DMI) outrank by domain power. Opportunity: clearer structure + visuals + freshness (2026 update) can win positions 4-8.</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>/blog/aeo-vs-geo-vs-seo/ — needs comparison table, simple 3-column visual, named author + bio. Schema: FAQPage + Article. Internal links from hub + both service pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>ai visibility consultant canada</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Local-intent SERP. Canadian + Toronto agencies + global GEO consultants.</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Chief AI Advisors (Victoria BC), dNOVO Group (Toronto), Pro Marketer (Canada), Semrush Toronto listings, Eric Schwartzman (US)</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Risk: dNOVO and Chief AI Advisors are direct Canadian competitors. Opportunity: personal-brand angle (Hami the person) is distinctive vs agency competitors.</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>/ai-visibility/ai-visibility-consultant-canada/ — emphasize personal brand (photo, bio, individual consultant not agency). Toronto-specific case study (HomeCalc fits — Canadian). Local schema, NAP, Google Business Profile if not done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>how to check ai visibility</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>380</v>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>SERP is DOMINATED BY FREE CHECKER TOOLS, not blog posts. Critical finding.</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Semrush free tool, Ubersuggest, Ahrefs, Amplitude, amivisibleonai.com, SEO Review Tools, SuSo Digital, Webtrek, LLMClicks, ResultFirst</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>MAJOR RISK: A pure how-to blog post likely will NOT rank for this query — Google is showing tools. Opportunity: pivot to 'tested these 10 checkers' listicle.</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>STRATEGIC PIVOT for /blog/how-to-check-ai-visibility/: reframe from 'how to check' instructional to 'I tested 10 free AI visibility checkers — here's what each found' listicle. Same URL, different angle. Ends with 'or skip the tools, get a real audit' CTA. OR: build a free checker tool eventually.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3753,7 +4024,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4303,7 +4574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add llms.txt for LLM site indexing
</commit_message>
<xml_diff>
--- a/master-seo-map.xlsx
+++ b/master-seo-map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dimah\hamitahm.com\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7AF915-A728-40CF-80BE-7A08CAD0CD68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076E1784-B279-488C-9F91-2576E049DD9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1327,7 +1327,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1400,6 +1400,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1428,7 +1434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1486,6 +1492,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1871,7 +1880,7 @@
       <c r="C2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="21" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="19" t="s">
@@ -1924,7 +1933,7 @@
       <c r="C3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="21" t="s">
         <v>31</v>
       </c>
       <c r="E3" s="19" t="s">
@@ -1977,7 +1986,7 @@
       <c r="C4" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="21" t="s">
         <v>42</v>
       </c>
       <c r="E4" s="19" t="s">
@@ -2030,7 +2039,7 @@
       <c r="C5" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="21" t="s">
         <v>51</v>
       </c>
       <c r="E5" s="19" t="s">
@@ -2083,7 +2092,7 @@
       <c r="C6" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="21" t="s">
         <v>61</v>
       </c>
       <c r="E6" s="19" t="s">
@@ -2136,7 +2145,7 @@
       <c r="C7" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="21" t="s">
         <v>69</v>
       </c>
       <c r="E7" s="19" t="s">
@@ -2189,7 +2198,7 @@
       <c r="C8" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="21" t="s">
         <v>77</v>
       </c>
       <c r="E8" s="19" t="s">
@@ -2242,7 +2251,7 @@
       <c r="C9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="21" t="s">
         <v>89</v>
       </c>
       <c r="E9" s="19" t="s">
@@ -2295,7 +2304,7 @@
       <c r="C10" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="21" t="s">
         <v>97</v>
       </c>
       <c r="E10" s="19" t="s">

</xml_diff>